<commit_message>
Excel de revisión y web de horarios (2026-10-29)
</commit_message>
<xml_diff>
--- a/data/horarios/Horarios_revision.xlsx
+++ b/data/horarios/Horarios_revision.xlsx
@@ -1,39 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cómo funciona" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Ciutat Vella" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Eixample" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Gràcia" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Horta-Guinardó" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Les Corts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Nou Barris" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Sant Andreu" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Sant Martí" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Sants-Montjuïc" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCN Sarrià-Sant Gervasi" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Badalona" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornellà de Llobregat" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L'Hospitalet de Llobregat" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mataró" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sant Adrià de Besòs" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Santa Coloma de Gramenet" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otros municipios" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Santuarios" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basílicas" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Iglesias" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capillas" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capillas de hospital" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capillas de residencia" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ermitas" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monasterios y conventos" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oratorios" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Cómo funciona" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BCN Ciutat Vella" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BCN Eixample" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="BCN Gràcia" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BCN Horta-Guinardó" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="BCN Les Corts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="BCN Nou Barris" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="BCN Sant Andreu" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="BCN Sant Martí" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="BCN Sants-Montjuïc" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="BCN Sarrià-Sant Gervasi" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Badalona" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Cornellà de Llobregat" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="L'Hospitalet de Llobregat" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Mataró" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Sant Adrià de Besòs" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Santa Coloma de Gramenet" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Otros municipios" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Santuarios" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Basílicas" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Iglesias" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Capillas" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Capillas de hospital" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Capillas de residencia" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Ermitas" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Monasterios y conventos" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Oratorios" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'BCN Ciutat Vella'!$A$1:$H$13</definedName>
@@ -14449,7 +14449,7 @@
       <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Misas: Lun–Vie 9:00, 10:00, 20:00; Sáb 9:00, 20:00; Dom y festivos 9:00, 10:30, 11:45, 13:00, 18:30, 20:00
-Adoración: Jue 20:30–22:30, 20:30–21:30</t>
+Adoración: Jue 20:30–21:30, 20:30–22:30</t>
         </is>
       </c>
       <c r="D7" s="9" t="n"/>
@@ -14550,7 +14550,7 @@
         <is>
           <t>Misas: Lun–Vie 9:00, 10:00, 20:00; Sáb 9:00, 20:00; Dom y festivos 9:00, 10:30, 11:45, 13:00, 18:30, 20:00
 Confesiones: antes de misa
-Adoración: Jue 20:30–22:30, 20:30–21:30</t>
+Adoración: Jue 20:30–21:30, 20:30–22:30</t>
         </is>
       </c>
       <c r="D10" s="9" t="n"/>
@@ -17598,9 +17598,9 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Misas: Lun–Sáb 20:00; Dom 11:30, 18:30, 20:00
-Confesiones: antes de misa
-Adoración: Vie 17:30</t>
+          <t>Misas: Lun–Vie 20:00; Sáb 20:00; Dom y festivos 11:30, 18:30, 20:00
+Confesiones: Mié 18:15–19:00; antes de misa
+Adoración: Vie 17:30–19:45</t>
         </is>
       </c>
       <c r="D7" s="9" t="n"/>
@@ -17610,7 +17610,7 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Arzobispado</t>
+          <t>Web propia</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">

</xml_diff>